<commit_message>
Aggiornata logica pipeline DDT: fotocopie, mappe mobile, distinte e conteggi
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/rientri_ddt.xlsx
+++ b/AppLogSolutionLocale/dati/rientri_ddt.xlsx
@@ -3,10 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Foglio1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.7265625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1774,9 +1775,351 @@
       </c>
     </row>
     <row r="91">
-      <c r="B91" s="1" t="n"/>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>p1736</t>
+        </is>
+      </c>
+      <c r="B91" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>p1752</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>p1754</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>p1755</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>p1759</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>p1761</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>p1762</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>p1764</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>p1765</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>p1766</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>p1788</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>p1808</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>p1816</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>p1831</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>p1892</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>p1902</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t>04/05/2026_2</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>p2176</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>p1788</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>p13474</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>p2428</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="n">
+        <v>46135</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[v1.54] Aggiornamenti Firebase rules e script logistica
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/rientri_ddt.xlsx
+++ b/AppLogSolutionLocale/dati/rientri_ddt.xlsx
@@ -1917,7 +1917,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 06-05-2026</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 06-05-2026</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,11 @@
       <c r="B107" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="C107" t="inlineStr"/>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2012,7 +2016,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 06-05-2026</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2031,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 06-05-2026</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2045,7 +2049,11 @@
       <c r="B110" s="1" t="n">
         <v>46135</v>
       </c>
-      <c r="C110" t="inlineStr"/>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
       <c r="D110" t="inlineStr">
         <is>
           <t>mancano 40 porzioni di mousse</t>
@@ -2063,7 +2071,11 @@
           <t>05-05-2026_FNS13695</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2076,7 +2088,11 @@
           <t>05-05-2026_FNS51851</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2089,7 +2105,11 @@
           <t>05-05-2026_FNS51848</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2102,7 +2122,11 @@
           <t>05-05-2026_FNS52172</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2115,7 +2139,11 @@
           <t>05-05-2026_FNS13653</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2128,7 +2156,11 @@
           <t>05-05-2026_FNS51831</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2143,7 +2175,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 06-05-2026</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2190,11 @@
           <t>05-05-2026_FNS52193</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2171,7 +2207,11 @@
           <t>05-05-2026_FNS51847</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2184,7 +2224,11 @@
           <t>05-05-2026_FNS51846</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2197,7 +2241,11 @@
           <t>05-05-2026_FNS51852</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2210,7 +2258,11 @@
           <t>05-05-2026_FNS51850</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2223,7 +2275,11 @@
           <t>05-05-2026_FNS51849</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2236,7 +2292,11 @@
           <t>05-05-2026_FNS51857</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2249,7 +2309,11 @@
           <t>05-05-2026_FNS13674</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2262,7 +2326,11 @@
           <t>05-05-2026_FNS13658</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2275,7 +2343,11 @@
           <t>05-05-2026_FNS13704</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>allegato DDT 06-05-2027</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[v2.8] Allineamento gestione rientri parziali e note
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/rientri_ddt.xlsx
+++ b/AppLogSolutionLocale/dati/rientri_ddt.xlsx
@@ -593,7 +593,6 @@
           <t>18-05-2026_FNS56443</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Tutto il ddt</t>
@@ -611,7 +610,6 @@
           <t>18-05-2026_FNS56468</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Tutto il ddt</t>
@@ -629,7 +627,6 @@
           <t>18-05-2026_FNS16051</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Tutto il ddt</t>
@@ -647,7 +644,6 @@
           <t>18-05-2026_FNS16047</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>parziale</t>
@@ -670,7 +666,6 @@
           <t>18-05-2026_FNS56167</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>parziale</t>
@@ -693,7 +688,6 @@
           <t>18-05-2026_FNS16097</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>parziale</t>
@@ -716,7 +710,6 @@
           <t>18-05-2026_FNS16049</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>parziale</t>
@@ -741,7 +734,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 20-05-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -768,7 +761,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 20-05-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -795,7 +788,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 20-05-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -822,7 +815,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 20-05-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -847,7 +840,6 @@
           <t>19-05-2026_FNS57255</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
[v2.8] Implementato visualizzatore nativo mappa_zone con editing interattivo e sync Firestore/Storage
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/rientri_ddt.xlsx
+++ b/AppLogSolutionLocale/dati/rientri_ddt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6216" yWindow="1476" windowWidth="23040" windowHeight="12120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7920" yWindow="1644" windowWidth="23040" windowHeight="12120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -848,6 +848,120 @@
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tutto il ddt</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>p1756</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13-04-2026_FNS9555</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>parziale</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>da consegnare 1 collo di grana padano</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>p2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13-05-2026_FNS15487</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tutto il ddt</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>p1850</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13-05-2026_FNS15450</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Tutto il ddt</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>p1791</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14-05-2026_FNS15670</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>allegato DDT 21-05-2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>parziale</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>da consegnare Latte intero alta qualità (fardello da 12 bottiglie) 1 fardello e 5 bottiglie</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>p8720</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>18-05-2026_FNS56989</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>parziale</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>da consegnare Mirtillo 1 collo e 4 porzioni</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Gestione dipendenti, sicurezza accessi e restyling icone commerciali/scuole nelle mappe
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/rientri_ddt.xlsx
+++ b/AppLogSolutionLocale/dati/rientri_ddt.xlsx
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 27-05-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 27-05-2026</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>in lavorazione</t>
+          <t>allegato DDT 27-05-2026</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1211,7 +1211,11 @@
           <t>25-05-2026_FNS59744</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>Tutto il ddt</t>
@@ -1229,7 +1233,11 @@
           <t>25-05-2026_FNS59743</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>In lavorazione</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Tutto il ddt</t>

</xml_diff>